<commit_message>
Update punctuation on gizmo file
The default type of apostrophe on LibreOffice doesnt work
Need to copy it from code?
</commit_message>
<xml_diff>
--- a/data/examples/gizmo_EDE.xlsx
+++ b/data/examples/gizmo_EDE.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
   <si>
     <t xml:space="preserve">EDE file for Gizmo</t>
   </si>
@@ -76,22 +76,16 @@
     <t xml:space="preserve">IP</t>
   </si>
   <si>
-    <t xml:space="preserve">DH’GF’Giz’AO4</t>
+    <t xml:space="preserve">DH'GF'Giz'AO4</t>
   </si>
   <si>
     <t xml:space="preserve">172.23.240.101</t>
   </si>
   <si>
-    <t xml:space="preserve">DH’GF’Giz’AI6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DH’GF’Giz’BO3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DH’GF’Giz’AI5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DH’GF’Giz’BI4</t>
+    <t xml:space="preserve">DH'GF'Giz'AI6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DH'GF'Giz'BO3</t>
   </si>
 </sst>
 </file>
@@ -106,6 +100,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -207,11 +202,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:R13"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="24.07"/>
@@ -221,7 +216,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="8.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="10.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="14.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="0" width="14.62"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="11.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="29.31"/>
@@ -300,7 +295,7 @@
       <c r="B9" s="0" t="n">
         <v>2098177</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="0" t="s">
         <v>18</v>
       </c>
       <c r="D9" s="0" t="n">
@@ -313,7 +308,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
         <v>20</v>
       </c>
@@ -333,7 +328,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="12.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
         <v>21</v>
       </c>
@@ -354,44 +349,20 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>2098177</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="R12" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="R12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>2098177</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="R13" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="R13" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>